<commit_message>
NR arreglado, mismo de Sora, mejores comentarios
</commit_message>
<xml_diff>
--- a/Proyecto_Python_Ver#2/Salida/Resultado.xlsx
+++ b/Proyecto_Python_Ver#2/Salida/Resultado.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="49">
   <si>
     <t>STATUS</t>
   </si>
@@ -63,24 +63,15 @@
     <t>ON</t>
   </si>
   <si>
-    <t>Bus 1</t>
-  </si>
-  <si>
-    <t>Bus 2</t>
-  </si>
-  <si>
-    <t>Bus 3</t>
-  </si>
-  <si>
     <t>SL</t>
   </si>
   <si>
+    <t>PV</t>
+  </si>
+  <si>
     <t>PQ</t>
   </si>
   <si>
-    <t>PV</t>
-  </si>
-  <si>
     <t>Bus j</t>
   </si>
   <si>
@@ -100,6 +91,18 @@
   </si>
   <si>
     <t>Line 3</t>
+  </si>
+  <si>
+    <t>Line 4</t>
+  </si>
+  <si>
+    <t>Line 5</t>
+  </si>
+  <si>
+    <t>Line 6</t>
+  </si>
+  <si>
+    <t>Line 7</t>
   </si>
   <si>
     <t>Xcc (pu)</t>
@@ -520,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -568,17 +571,17 @@
       <c r="A2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>17</v>
-      </c>
       <c r="E2">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -602,22 +605,22 @@
         <v>0</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
       <c r="E3">
         <v>1</v>
       </c>
@@ -625,16 +628,16 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I3">
-        <v>4</v>
+        <v>0.2</v>
       </c>
       <c r="J3">
-        <v>2.5</v>
+        <v>0.1</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -643,39 +646,39 @@
         <v>0</v>
       </c>
       <c r="M3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
-        <v>16</v>
+      <c r="B4">
+        <v>3</v>
       </c>
       <c r="C4">
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E4">
-        <v>1.04</v>
+        <v>1</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -684,7 +687,89 @@
         <v>0</v>
       </c>
       <c r="M4">
-        <v>0</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0.4</v>
+      </c>
+      <c r="J5">
+        <v>0.05</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0.6</v>
+      </c>
+      <c r="J6">
+        <v>0.1</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -694,7 +779,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -708,16 +793,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -725,7 +810,7 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -737,7 +822,7 @@
         <v>0.02</v>
       </c>
       <c r="F2">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -748,7 +833,7 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -757,13 +842,13 @@
         <v>3</v>
       </c>
       <c r="E3">
-        <v>0.01</v>
+        <v>0.08</v>
       </c>
       <c r="F3">
-        <v>0.03</v>
+        <v>0.24</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -771,7 +856,7 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -780,13 +865,105 @@
         <v>3</v>
       </c>
       <c r="E4">
-        <v>0.0125</v>
+        <v>0.06</v>
       </c>
       <c r="F4">
+        <v>0.25</v>
+      </c>
+      <c r="G4">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>0.06</v>
+      </c>
+      <c r="F5">
+        <v>0.18</v>
+      </c>
+      <c r="G5">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>0.04</v>
+      </c>
+      <c r="F6">
+        <v>0.12</v>
+      </c>
+      <c r="G6">
+        <v>0.015</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>0.01</v>
+      </c>
+      <c r="F7">
+        <v>0.03</v>
+      </c>
+      <c r="G7">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8">
+        <v>4</v>
+      </c>
+      <c r="D8">
+        <v>5</v>
+      </c>
+      <c r="E8">
+        <v>0.08</v>
+      </c>
+      <c r="F8">
+        <v>0.24</v>
+      </c>
+      <c r="G8">
         <v>0.025</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -810,16 +987,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -843,10 +1020,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -856,21 +1033,21 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B1">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D1">
-        <v>9.219655662375597E-05</v>
+        <v>7.950549010655649E-05</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -878,51 +1055,51 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>14</v>
+      <c r="A3">
+        <v>1</v>
       </c>
       <c r="B3">
-        <v>1.05</v>
+        <v>1.06</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>2.1812</v>
+        <v>4.0213</v>
       </c>
       <c r="E3">
-        <v>1.4095</v>
+        <v>8.176299999999999</v>
       </c>
       <c r="F3">
-        <v>2.1812</v>
+        <v>4.0213</v>
       </c>
       <c r="G3">
-        <v>1.4095</v>
+        <v>8.176299999999999</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -932,61 +1109,119 @@
       </c>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>15</v>
+      <c r="A4">
+        <v>2</v>
       </c>
       <c r="B4">
-        <v>0.9717</v>
+        <v>1</v>
       </c>
       <c r="C4">
-        <v>-2.6927</v>
+        <v>-3.2001</v>
       </c>
       <c r="D4">
-        <v>-4</v>
+        <v>0.2</v>
       </c>
       <c r="E4">
-        <v>-2.5</v>
+        <v>1.3892</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1.4892</v>
       </c>
       <c r="H4">
+        <v>0.2</v>
+      </c>
+      <c r="I4">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>0.3174</v>
+      </c>
+      <c r="C5">
+        <v>-23.2939</v>
+      </c>
+      <c r="D5">
+        <v>-0.45</v>
+      </c>
+      <c r="E5">
+        <v>-0.15</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0.45</v>
+      </c>
+      <c r="I5">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6">
         <v>4</v>
       </c>
-      <c r="I4">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5">
-        <v>1.04</v>
-      </c>
-      <c r="C5">
-        <v>-0.496</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5">
-        <v>1.4613</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>1.4613</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
+      <c r="B6">
+        <v>1.2148</v>
+      </c>
+      <c r="C6">
+        <v>-5.6023</v>
+      </c>
+      <c r="D6">
+        <v>-0.4</v>
+      </c>
+      <c r="E6">
+        <v>-0.05</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>0.4</v>
+      </c>
+      <c r="I6">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>1.387</v>
+      </c>
+      <c r="C7">
+        <v>-5.2281</v>
+      </c>
+      <c r="D7">
+        <v>-0.6</v>
+      </c>
+      <c r="E7">
+        <v>-0.1</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0.6</v>
+      </c>
+      <c r="I7">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -996,41 +1231,41 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1039,27 +1274,27 @@
         <v>2</v>
       </c>
       <c r="D2">
-        <v>1.7922</v>
+        <v>1.2139</v>
       </c>
       <c r="E2">
-        <v>1.1878</v>
+        <v>0.6829</v>
       </c>
       <c r="F2">
-        <v>-1.7083</v>
+        <v>-1.1793</v>
       </c>
       <c r="G2">
-        <v>-1.0201</v>
+        <v>-0.5918</v>
       </c>
       <c r="H2">
-        <v>0.0839</v>
+        <v>0.0345</v>
       </c>
       <c r="I2">
-        <v>0.1677</v>
+        <v>0.0911</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1068,27 +1303,27 @@
         <v>3</v>
       </c>
       <c r="D3">
-        <v>0.389</v>
+        <v>1.5172</v>
       </c>
       <c r="E3">
-        <v>0.2217</v>
+        <v>2.8883</v>
       </c>
       <c r="F3">
-        <v>-0.3872</v>
+        <v>-0.7593</v>
       </c>
       <c r="G3">
-        <v>-0.2162</v>
+        <v>-0.6158</v>
       </c>
       <c r="H3">
-        <v>0.0018</v>
+        <v>0.7579</v>
       </c>
       <c r="I3">
-        <v>0.0055</v>
+        <v>2.2725</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -1097,22 +1332,138 @@
         <v>3</v>
       </c>
       <c r="D4">
-        <v>-2.2897</v>
+        <v>1.0496</v>
       </c>
       <c r="E4">
-        <v>-1.4807</v>
+        <v>2.5432</v>
       </c>
       <c r="F4">
-        <v>2.3881</v>
+        <v>-0.5916</v>
       </c>
       <c r="G4">
-        <v>1.6776</v>
+        <v>-0.6484</v>
       </c>
       <c r="H4">
-        <v>0.0984</v>
+        <v>0.458</v>
       </c>
       <c r="I4">
-        <v>0.1969</v>
+        <v>1.8948</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>-0.1017</v>
+      </c>
+      <c r="E5">
+        <v>-1.1662</v>
+      </c>
+      <c r="F5">
+        <v>0.1822</v>
+      </c>
+      <c r="G5">
+        <v>1.3804</v>
+      </c>
+      <c r="H5">
+        <v>0.0805</v>
+      </c>
+      <c r="I5">
+        <v>0.2142</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>-0.5972</v>
+      </c>
+      <c r="E6">
+        <v>-3.0312</v>
+      </c>
+      <c r="F6">
+        <v>0.976</v>
+      </c>
+      <c r="G6">
+        <v>4.1405</v>
+      </c>
+      <c r="H6">
+        <v>0.3788</v>
+      </c>
+      <c r="I6">
+        <v>1.1094</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7">
+        <v>-6.1817</v>
+      </c>
+      <c r="E7">
+        <v>-6.8278</v>
+      </c>
+      <c r="F7">
+        <v>14.6002</v>
+      </c>
+      <c r="G7">
+        <v>32.0674</v>
+      </c>
+      <c r="H7">
+        <v>8.4185</v>
+      </c>
+      <c r="I7">
+        <v>25.2396</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8">
+        <v>-0.3026</v>
+      </c>
+      <c r="E8">
+        <v>-0.7852</v>
+      </c>
+      <c r="F8">
+        <v>0.3398</v>
+      </c>
+      <c r="G8">
+        <v>0.8673999999999999</v>
+      </c>
+      <c r="H8">
+        <v>0.0371</v>
+      </c>
+      <c r="I8">
+        <v>0.0822</v>
       </c>
     </row>
   </sheetData>

</xml_diff>